<commit_message>
Logo en Reporte de Honorarios
</commit_message>
<xml_diff>
--- a/templates/PlantillaReporte.xlsx
+++ b/templates/PlantillaReporte.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F4AE939D-A58C-4722-AE99-FBB61E74174E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{02BD88F9-F43B-47C5-92AC-3FBE21E3D2EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -606,15 +606,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>276225</xdr:colOff>
+      <xdr:colOff>371475</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>161925</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -637,8 +637,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="276225" y="247650"/>
-          <a:ext cx="3171825" cy="552450"/>
+          <a:off x="371475" y="238125"/>
+          <a:ext cx="2047875" cy="733425"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>